<commit_message>
New model (MC); update columns, include new distribution.
</commit_message>
<xml_diff>
--- a/api/Modelo_Riscos.xlsx
+++ b/api/Modelo_Riscos.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Crucialidade Atividades" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Crucialidade Caminhos" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Distribuição Projeto e Risco" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Custos" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,28 +494,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>9.183172533460752</v>
+        <v>6.436250505455263</v>
       </c>
       <c r="C2" t="n">
-        <v>11.81131767582138</v>
+        <v>7.141636595157508</v>
       </c>
       <c r="D2" t="n">
-        <v>3.889758189114261</v>
+        <v>2.389752171239094</v>
       </c>
       <c r="E2" t="n">
-        <v>6.197962889691848</v>
+        <v>6.119323018688289</v>
       </c>
       <c r="F2" t="n">
-        <v>10.32697358089793</v>
+        <v>9.119028564387763</v>
       </c>
       <c r="G2" t="n">
-        <v>4.03419954230521</v>
+        <v>4.888755656308191</v>
       </c>
       <c r="H2" t="n">
-        <v>8.693216772581069</v>
+        <v>8.264987073071303</v>
       </c>
       <c r="I2" t="n">
-        <v>4.548626302011878</v>
+        <v>5.077496848449548</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -525,28 +526,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>5.376673276062931</v>
+        <v>8.680379676662806</v>
       </c>
       <c r="C3" t="n">
-        <v>7.93506093902411</v>
+        <v>6.887808177115594</v>
       </c>
       <c r="D3" t="n">
-        <v>3.034532687380171</v>
+        <v>2.545271706573525</v>
       </c>
       <c r="E3" t="n">
-        <v>6.173989674282716</v>
+        <v>6.132467842337074</v>
       </c>
       <c r="F3" t="n">
-        <v>9.964932314182899</v>
+        <v>9.067106155172391</v>
       </c>
       <c r="G3" t="n">
-        <v>5.468599525049587</v>
+        <v>4.05706034490938</v>
       </c>
       <c r="H3" t="n">
-        <v>7.194562306207124</v>
+        <v>8.397565661974422</v>
       </c>
       <c r="I3" t="n">
-        <v>3.991905850917887</v>
+        <v>5.17683672507288</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -557,28 +558,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>4.188604249466144</v>
+        <v>4.790259968486747</v>
       </c>
       <c r="C4" t="n">
-        <v>9.376480437732759</v>
+        <v>5.725827175958816</v>
       </c>
       <c r="D4" t="n">
-        <v>2.091708621650965</v>
+        <v>2.253171526432489</v>
       </c>
       <c r="E4" t="n">
-        <v>5.664663845766603</v>
+        <v>5.457800684949743</v>
       </c>
       <c r="F4" t="n">
-        <v>9.726314974244884</v>
+        <v>9.72517047473931</v>
       </c>
       <c r="G4" t="n">
-        <v>5.126337684998758</v>
+        <v>4.486181200413191</v>
       </c>
       <c r="H4" t="n">
-        <v>9.419055895434237</v>
+        <v>7.860640762161255</v>
       </c>
       <c r="I4" t="n">
-        <v>4.141664494018262</v>
+        <v>5.554642916019329</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -589,28 +590,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>4.227393988065401</v>
+        <v>8.678870542201818</v>
       </c>
       <c r="C5" t="n">
-        <v>5.075260839902766</v>
+        <v>8.368000135160932</v>
       </c>
       <c r="D5" t="n">
-        <v>2.613789294278628</v>
+        <v>2.259766436922458</v>
       </c>
       <c r="E5" t="n">
-        <v>6.271003357263905</v>
+        <v>5.895164262322868</v>
       </c>
       <c r="F5" t="n">
-        <v>10.28779413328161</v>
+        <v>9.673663681228309</v>
       </c>
       <c r="G5" t="n">
-        <v>5.392550030033493</v>
+        <v>4.552078986211999</v>
       </c>
       <c r="H5" t="n">
-        <v>7.469510185464431</v>
+        <v>8.354179874102002</v>
       </c>
       <c r="I5" t="n">
-        <v>5.669900214993887</v>
+        <v>5.779788889138638</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -621,31 +622,262 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>7.569368688893255</v>
+        <v>7.630842786081775</v>
       </c>
       <c r="C6" t="n">
-        <v>7.700652010443251</v>
+        <v>9.643020923994895</v>
       </c>
       <c r="D6" t="n">
-        <v>1.049389992855227</v>
+        <v>2.782810335183619</v>
       </c>
       <c r="E6" t="n">
-        <v>5.871739166767611</v>
+        <v>5.580991686738384</v>
       </c>
       <c r="F6" t="n">
-        <v>10.43612673045522</v>
+        <v>11.26900400108408</v>
       </c>
       <c r="G6" t="n">
-        <v>5.357022011831405</v>
+        <v>3.990758692061747</v>
       </c>
       <c r="H6" t="n">
-        <v>7.969608163377076</v>
+        <v>7.517015754056018</v>
       </c>
       <c r="I6" t="n">
-        <v>4.215443095011127</v>
+        <v>5.060503016714734</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>10.94515772938654</v>
+      </c>
+      <c r="C7" t="n">
+        <v>7.722683480556348</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.864638550189972</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.827926232471811</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10.60962444641179</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5.555490481024819</v>
+      </c>
+      <c r="H7" t="n">
+        <v>9.632512462502495</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.544635791695613</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>8.574988239550267</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7.643423243681644</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.56465334639511</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6.244187102153069</v>
+      </c>
+      <c r="F8" t="n">
+        <v>9.043009209907645</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.700601827116669</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7.530802427672416</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.872425294488211</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8.367775547170359</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10.38230642639892</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.706197319289919</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.009834218315729</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11.65581208150017</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.532865444682809</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7.09388459082566</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.625986652809063</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9.541954610626881</v>
+      </c>
+      <c r="C10" t="n">
+        <v>11.84352926282863</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4.728872483643938</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.931608037505933</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10.76511114132571</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.538803745032144</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8.274201215552782</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.987519253030357</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>9.865520475794096</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5.630862214431534</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.108732735604447</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5.609197371157459</v>
+      </c>
+      <c r="F11" t="n">
+        <v>8.772046304236389</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5.531577618132238</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9.164127523683593</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.962278796368707</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Custos por Iteração</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>112.6723149944753</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>115.5680619159471</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>110.0361916836467</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>115.8060005591795</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>114.4683012948642</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>118.8653294833086</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>115.4311672661168</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>115.5753132584295</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>117.624285942722</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>116.9060140403868</v>
       </c>
     </row>
   </sheetData>
@@ -659,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,13 +921,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>24.07047667710255</v>
+        <v>25.9338917766096</v>
       </c>
       <c r="C2" t="n">
-        <v>41.58412599605803</v>
+        <v>27.96219719237236</v>
       </c>
       <c r="D2" t="n">
-        <v>30.80477106058809</v>
+        <v>17.38401563745906</v>
       </c>
     </row>
     <row r="3">
@@ -703,13 +935,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>33.56122224889264</v>
+        <v>27.34735663033419</v>
       </c>
       <c r="C3" t="n">
-        <v>38.23142866509864</v>
+        <v>30.0982213580899</v>
       </c>
       <c r="D3" t="n">
-        <v>28.9810805537519</v>
+        <v>17.46467181714682</v>
       </c>
     </row>
     <row r="4">
@@ -717,13 +949,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>34.27245132083585</v>
+        <v>22.81008278731057</v>
       </c>
       <c r="C4" t="n">
-        <v>41.81669097747347</v>
+        <v>23.83452859155656</v>
       </c>
       <c r="D4" t="n">
-        <v>30.85769496207571</v>
+        <v>17.58581123690056</v>
       </c>
     </row>
     <row r="5">
@@ -731,13 +963,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>26.75871358430776</v>
+        <v>29.63850498963584</v>
       </c>
       <c r="C5" t="n">
-        <v>30.17794005456167</v>
+        <v>31.29621481378762</v>
       </c>
       <c r="D5" t="n">
-        <v>20.85761148782163</v>
+        <v>18.02784355533031</v>
       </c>
     </row>
     <row r="6">
@@ -745,13 +977,83 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>23.87358717326249</v>
+        <v>29.10793575403677</v>
       </c>
       <c r="C6" t="n">
-        <v>33.6757555931688</v>
+        <v>30.37187115087107</v>
       </c>
       <c r="D6" t="n">
-        <v>24.95288428284101</v>
+        <v>18.7860197551401</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>30.63260603285329</v>
+      </c>
+      <c r="C7" t="n">
+        <v>34.12827990491719</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20.24213690891428</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>27.3560919512319</v>
+      </c>
+      <c r="C8" t="n">
+        <v>29.9934010130574</v>
+      </c>
+      <c r="D8" t="n">
+        <v>16.57381163758006</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>29.61513139035107</v>
+      </c>
+      <c r="C9" t="n">
+        <v>31.85380078271067</v>
+      </c>
+      <c r="D9" t="n">
+        <v>18.74969667232583</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>35.64067935516196</v>
+      </c>
+      <c r="C10" t="n">
+        <v>35.59129312651423</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19.0393123568785</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>27.09897184033102</v>
+      </c>
+      <c r="C11" t="n">
+        <v>30.26970758506668</v>
+      </c>
+      <c r="D11" t="n">
+        <v>17.93617382791998</v>
       </c>
     </row>
   </sheetData>
@@ -765,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +1098,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>['start', 1, 2, 5, 7, 'end']</t>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -805,7 +1107,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>41.58412599605803</v>
+        <v>27.96219719237236</v>
       </c>
     </row>
     <row r="3">
@@ -814,7 +1116,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>['start', 1, 2, 5, 7, 'end']</t>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -823,7 +1125,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>38.23142866509864</v>
+        <v>30.0982213580899</v>
       </c>
     </row>
     <row r="4">
@@ -832,7 +1134,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>['start', 1, 2, 5, 7, 'end']</t>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -841,7 +1143,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>41.81669097747347</v>
+        <v>23.83452859155656</v>
       </c>
     </row>
     <row r="5">
@@ -850,7 +1152,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>['start', 1, 2, 5, 7, 'end']</t>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -859,7 +1161,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>30.17794005456167</v>
+        <v>31.29621481378762</v>
       </c>
     </row>
     <row r="6">
@@ -868,7 +1170,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>['start', 1, 2, 5, 7, 'end']</t>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -877,7 +1179,97 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>33.6757555931688</v>
+        <v>30.37187115087107</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Caminho 2</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>34.12827990491719</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Caminho 2</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>29.9934010130574</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Caminho 2</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>31.85380078271067</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>['start', 1, 2, 3, 6, 8, 'end']</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Caminho 1</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>35.64067935516196</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>['start', 1, 2, 4, 7, 'end']</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Caminho 2</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>30.26970758506668</v>
       </c>
     </row>
   </sheetData>
@@ -891,7 +1283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,12 +1311,12 @@
         <v>1</v>
       </c>
       <c r="B3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" t="b">
         <v>0</v>
@@ -940,10 +1332,10 @@
     </row>
     <row r="6">
       <c r="A6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -959,12 +1351,12 @@
         <v>1</v>
       </c>
       <c r="B8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="b">
         <v>1</v>
@@ -975,54 +1367,14 @@
         <v>1</v>
       </c>
       <c r="B10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="b">
-        <v>0</v>
-      </c>
-      <c r="B12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="b">
-        <v>0</v>
-      </c>
-      <c r="B13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="b">
-        <v>0</v>
-      </c>
-      <c r="B14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1068,14 +1420,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>('start', 1, 2, 4, 7, 'end')</t>
+          <t>('start', 1, 2, 3, 6, 8, 'end')</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
@@ -1084,14 +1436,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>('start', 1, 2, 5, 7, 'end')</t>
+          <t>('start', 1, 2, 4, 7, 'end')</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4">
@@ -1100,7 +1452,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>('start', 1, 3, 6, 8, 'end')</t>
+          <t>('start', 5, 7, 'end')</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1148,7 +1500,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -1161,7 +1513,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -1174,10 +1526,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -1187,10 +1539,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6">
@@ -1200,10 +1552,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1213,10 +1565,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8">
@@ -1226,10 +1578,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
@@ -1239,10 +1591,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
@@ -1252,7 +1604,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -1291,7 +1643,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2667166292031236</v>
+        <v>0.86529151901201</v>
       </c>
     </row>
     <row r="3">
@@ -1301,7 +1653,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8931118552806936</v>
+        <v>0.6974713724972444</v>
       </c>
     </row>
     <row r="4">
@@ -1311,7 +1663,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4219522386525625</v>
+        <v>0.3667176463948956</v>
       </c>
     </row>
     <row r="5">
@@ -1321,7 +1673,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.3693014838274717</v>
+        <v>0.3010376872811633</v>
       </c>
     </row>
     <row r="6">
@@ -1331,7 +1683,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.5601125120946908</v>
+        <v>0.4415299220009342</v>
       </c>
     </row>
     <row r="7">
@@ -1341,7 +1693,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.5896323169702961</v>
+        <v>0.1993303455020391</v>
       </c>
     </row>
     <row r="8">
@@ -1351,7 +1703,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6847842754997787</v>
+        <v>0.2884992148835177</v>
       </c>
     </row>
     <row r="9">
@@ -1361,7 +1713,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.6656782044585176</v>
+        <v>-0.3217009819547498</v>
       </c>
     </row>
     <row r="10">
@@ -1403,31 +1755,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>('start', 1, 2, 4, 7, 'end')</t>
+          <t>('start', 1, 2, 3, 6, 8, 'end')</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3974059547918108</v>
+        <v>0.9485208511182573</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>('start', 1, 2, 5, 7, 'end')</t>
+          <t>('start', 1, 2, 4, 7, 'end')</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.9999918348357516</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>('start', 1, 3, 6, 8, 'end')</t>
+          <t>('start', 5, 7, 'end')</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9903297143263607</v>
+        <v>0.6467705383759255</v>
       </c>
     </row>
   </sheetData>
@@ -1441,7 +1793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1453,27 +1805,52 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>41.58412599605803</v>
+        <v>27.96219719237236</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>38.23142866509864</v>
+        <v>30.0982213580899</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>41.81669097747347</v>
+        <v>23.83452859155656</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>30.17794005456167</v>
+        <v>31.29621481378762</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>33.6757555931688</v>
+        <v>30.37187115087107</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>34.12827990491719</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>29.9934010130574</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>31.85380078271067</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>35.64067935516196</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>30.26970758506668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>